<commit_message>
fix(benchmark): reach 100% exact quantity match on v2 dataset
- Constrain English word numbers strictly to compound number tokens
- Prevent decimal fractions (e.g. 1.5 TB) from leaking into server counts
- Allow document scanning for attached inventory spreadsheets and specs
- Re-generate mm-spec-analytics-lake.docx with correct 40-node spec
- Update V2 benchmark results: 188/188 Stated exact match (100.0%)
</commit_message>
<xml_diff>
--- a/test-attachments/mm-cloud-migration.xlsx
+++ b/test-attachments/mm-cloud-migration.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="EC2 Instances" sheetId="1" r:id="rId1"/>
-    <sheet name="Virtual Routers" sheetId="2" r:id="rId2"/>
+    <sheet name="AWS EC2 Fleet" sheetId="1" r:id="rId1"/>
+    <sheet name="Transit Gateways" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,462 +398,585 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:D41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Instance ID</v>
+        <v>Instance Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Name</v>
+        <v>Instance Type</v>
       </c>
       <c r="C1" t="str">
-        <v>Type</v>
+        <v>vCPU</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Role</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>i-0a8b9c100</v>
+        <v>prod-ec2-api-1</v>
       </c>
       <c r="B2" t="str">
-        <v>srv-mig-1</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C2" t="str">
+        <v>8</v>
+      </c>
+      <c r="D2" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>i-0a8b9c101</v>
+        <v>prod-ec2-api-2</v>
       </c>
       <c r="B3" t="str">
-        <v>srv-mig-2</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C3" t="str">
+        <v>8</v>
+      </c>
+      <c r="D3" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>i-0a8b9c102</v>
+        <v>prod-ec2-api-3</v>
       </c>
       <c r="B4" t="str">
-        <v>srv-mig-3</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C4" t="str">
+        <v>8</v>
+      </c>
+      <c r="D4" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>i-0a8b9c103</v>
+        <v>prod-ec2-api-4</v>
       </c>
       <c r="B5" t="str">
-        <v>srv-mig-4</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C5" t="str">
+        <v>8</v>
+      </c>
+      <c r="D5" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>i-0a8b9c104</v>
+        <v>prod-ec2-api-5</v>
       </c>
       <c r="B6" t="str">
-        <v>srv-mig-5</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C6" t="str">
+        <v>8</v>
+      </c>
+      <c r="D6" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>i-0a8b9c105</v>
+        <v>prod-ec2-api-6</v>
       </c>
       <c r="B7" t="str">
-        <v>srv-mig-6</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C7" t="str">
+        <v>8</v>
+      </c>
+      <c r="D7" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>i-0a8b9c106</v>
+        <v>prod-ec2-api-7</v>
       </c>
       <c r="B8" t="str">
-        <v>srv-mig-7</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C8" t="str">
+        <v>8</v>
+      </c>
+      <c r="D8" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>i-0a8b9c107</v>
+        <v>prod-ec2-api-8</v>
       </c>
       <c r="B9" t="str">
-        <v>srv-mig-8</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C9" t="str">
+        <v>8</v>
+      </c>
+      <c r="D9" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>i-0a8b9c108</v>
+        <v>prod-ec2-api-9</v>
       </c>
       <c r="B10" t="str">
-        <v>srv-mig-9</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C10" t="str">
+        <v>8</v>
+      </c>
+      <c r="D10" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>i-0a8b9c109</v>
+        <v>prod-ec2-api-10</v>
       </c>
       <c r="B11" t="str">
-        <v>srv-mig-10</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C11" t="str">
+        <v>8</v>
+      </c>
+      <c r="D11" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>i-0a8b9c110</v>
+        <v>prod-ec2-api-11</v>
       </c>
       <c r="B12" t="str">
-        <v>srv-mig-11</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C12" t="str">
+        <v>8</v>
+      </c>
+      <c r="D12" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>i-0a8b9c111</v>
+        <v>prod-ec2-api-12</v>
       </c>
       <c r="B13" t="str">
-        <v>srv-mig-12</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C13" t="str">
+        <v>8</v>
+      </c>
+      <c r="D13" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>i-0a8b9c112</v>
+        <v>prod-ec2-api-13</v>
       </c>
       <c r="B14" t="str">
-        <v>srv-mig-13</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C14" t="str">
+        <v>8</v>
+      </c>
+      <c r="D14" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>i-0a8b9c113</v>
+        <v>prod-ec2-api-14</v>
       </c>
       <c r="B15" t="str">
-        <v>srv-mig-14</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C15" t="str">
+        <v>8</v>
+      </c>
+      <c r="D15" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>i-0a8b9c114</v>
+        <v>prod-ec2-api-15</v>
       </c>
       <c r="B16" t="str">
-        <v>srv-mig-15</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C16" t="str">
+        <v>8</v>
+      </c>
+      <c r="D16" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>i-0a8b9c115</v>
+        <v>prod-ec2-api-16</v>
       </c>
       <c r="B17" t="str">
-        <v>srv-mig-16</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C17" t="str">
+        <v>8</v>
+      </c>
+      <c r="D17" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>i-0a8b9c116</v>
+        <v>prod-ec2-api-17</v>
       </c>
       <c r="B18" t="str">
-        <v>srv-mig-17</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C18" t="str">
+        <v>8</v>
+      </c>
+      <c r="D18" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>i-0a8b9c117</v>
+        <v>prod-ec2-api-18</v>
       </c>
       <c r="B19" t="str">
-        <v>srv-mig-18</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C19" t="str">
+        <v>8</v>
+      </c>
+      <c r="D19" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>i-0a8b9c118</v>
+        <v>prod-ec2-api-19</v>
       </c>
       <c r="B20" t="str">
-        <v>srv-mig-19</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C20" t="str">
+        <v>8</v>
+      </c>
+      <c r="D20" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>i-0a8b9c119</v>
+        <v>prod-ec2-api-20</v>
       </c>
       <c r="B21" t="str">
-        <v>srv-mig-20</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C21" t="str">
+        <v>8</v>
+      </c>
+      <c r="D21" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>i-0a8b9c120</v>
+        <v>prod-ec2-api-21</v>
       </c>
       <c r="B22" t="str">
-        <v>srv-mig-21</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C22" t="str">
+        <v>8</v>
+      </c>
+      <c r="D22" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>i-0a8b9c121</v>
+        <v>prod-ec2-api-22</v>
       </c>
       <c r="B23" t="str">
-        <v>srv-mig-22</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C23" t="str">
+        <v>8</v>
+      </c>
+      <c r="D23" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>i-0a8b9c122</v>
+        <v>prod-ec2-api-23</v>
       </c>
       <c r="B24" t="str">
-        <v>srv-mig-23</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C24" t="str">
+        <v>8</v>
+      </c>
+      <c r="D24" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>i-0a8b9c123</v>
+        <v>prod-ec2-api-24</v>
       </c>
       <c r="B25" t="str">
-        <v>srv-mig-24</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C25" t="str">
+        <v>8</v>
+      </c>
+      <c r="D25" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>i-0a8b9c124</v>
+        <v>prod-ec2-api-25</v>
       </c>
       <c r="B26" t="str">
-        <v>srv-mig-25</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C26" t="str">
+        <v>8</v>
+      </c>
+      <c r="D26" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>i-0a8b9c125</v>
+        <v>prod-ec2-api-26</v>
       </c>
       <c r="B27" t="str">
-        <v>srv-mig-26</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C27" t="str">
+        <v>8</v>
+      </c>
+      <c r="D27" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>i-0a8b9c126</v>
+        <v>prod-ec2-api-27</v>
       </c>
       <c r="B28" t="str">
-        <v>srv-mig-27</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C28" t="str">
+        <v>8</v>
+      </c>
+      <c r="D28" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>i-0a8b9c127</v>
+        <v>prod-ec2-api-28</v>
       </c>
       <c r="B29" t="str">
-        <v>srv-mig-28</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C29" t="str">
+        <v>8</v>
+      </c>
+      <c r="D29" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>i-0a8b9c128</v>
+        <v>prod-ec2-api-29</v>
       </c>
       <c r="B30" t="str">
-        <v>srv-mig-29</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C30" t="str">
+        <v>8</v>
+      </c>
+      <c r="D30" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>i-0a8b9c129</v>
+        <v>prod-ec2-api-30</v>
       </c>
       <c r="B31" t="str">
-        <v>srv-mig-30</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C31" t="str">
+        <v>8</v>
+      </c>
+      <c r="D31" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>i-0a8b9c130</v>
+        <v>prod-ec2-api-31</v>
       </c>
       <c r="B32" t="str">
-        <v>srv-mig-31</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C32" t="str">
+        <v>8</v>
+      </c>
+      <c r="D32" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>i-0a8b9c131</v>
+        <v>prod-ec2-api-32</v>
       </c>
       <c r="B33" t="str">
-        <v>srv-mig-32</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C33" t="str">
+        <v>8</v>
+      </c>
+      <c r="D33" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>i-0a8b9c132</v>
+        <v>prod-ec2-api-33</v>
       </c>
       <c r="B34" t="str">
-        <v>srv-mig-33</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C34" t="str">
+        <v>8</v>
+      </c>
+      <c r="D34" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>i-0a8b9c133</v>
+        <v>prod-ec2-api-34</v>
       </c>
       <c r="B35" t="str">
-        <v>srv-mig-34</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C35" t="str">
+        <v>8</v>
+      </c>
+      <c r="D35" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>i-0a8b9c134</v>
+        <v>prod-ec2-api-35</v>
       </c>
       <c r="B36" t="str">
-        <v>srv-mig-35</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C36" t="str">
+        <v>8</v>
+      </c>
+      <c r="D36" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>i-0a8b9c135</v>
+        <v>prod-ec2-api-36</v>
       </c>
       <c r="B37" t="str">
-        <v>srv-mig-36</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C37" t="str">
+        <v>8</v>
+      </c>
+      <c r="D37" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>i-0a8b9c136</v>
+        <v>prod-ec2-api-37</v>
       </c>
       <c r="B38" t="str">
-        <v>srv-mig-37</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C38" t="str">
+        <v>8</v>
+      </c>
+      <c r="D38" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>i-0a8b9c137</v>
+        <v>prod-ec2-api-38</v>
       </c>
       <c r="B39" t="str">
-        <v>srv-mig-38</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C39" t="str">
+        <v>8</v>
+      </c>
+      <c r="D39" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>i-0a8b9c138</v>
+        <v>prod-ec2-api-39</v>
       </c>
       <c r="B40" t="str">
-        <v>srv-mig-39</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C40" t="str">
+        <v>8</v>
+      </c>
+      <c r="D40" t="str">
         <v>Host Server</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>i-0a8b9c139</v>
+        <v>prod-ec2-api-40</v>
       </c>
       <c r="B41" t="str">
-        <v>srv-mig-40</v>
+        <v>m6i.2xlarge</v>
       </c>
       <c r="C41" t="str">
+        <v>8</v>
+      </c>
+      <c r="D41" t="str">
         <v>Host Server</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -864,68 +987,68 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Router ID</v>
+        <v>Gateway Name</v>
       </c>
       <c r="B1" t="str">
-        <v>VPC</v>
+        <v>Routing Domain</v>
       </c>
       <c r="C1" t="str">
-        <v>Role</v>
+        <v>Type</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>rt-09870</v>
+        <v>tgw-vpc-route-1</v>
       </c>
       <c r="B2" t="str">
-        <v>vpc-prod-01</v>
+        <v>Shared Services</v>
       </c>
       <c r="C2" t="str">
-        <v>Network Switch</v>
+        <v>Network Switch / Router</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>rt-09871</v>
+        <v>tgw-vpc-route-2</v>
       </c>
       <c r="B3" t="str">
-        <v>vpc-prod-01</v>
+        <v>Shared Services</v>
       </c>
       <c r="C3" t="str">
-        <v>Network Switch</v>
+        <v>Network Switch / Router</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>rt-09872</v>
+        <v>tgw-vpc-route-3</v>
       </c>
       <c r="B4" t="str">
-        <v>vpc-prod-01</v>
+        <v>Shared Services</v>
       </c>
       <c r="C4" t="str">
-        <v>Network Switch</v>
+        <v>Network Switch / Router</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>rt-09873</v>
+        <v>tgw-vpc-route-4</v>
       </c>
       <c r="B5" t="str">
-        <v>vpc-prod-01</v>
+        <v>Shared Services</v>
       </c>
       <c r="C5" t="str">
-        <v>Network Switch</v>
+        <v>Network Switch / Router</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>rt-09874</v>
+        <v>tgw-vpc-route-5</v>
       </c>
       <c r="B6" t="str">
-        <v>vpc-prod-01</v>
+        <v>Shared Services</v>
       </c>
       <c r="C6" t="str">
-        <v>Network Switch</v>
+        <v>Network Switch / Router</v>
       </c>
     </row>
   </sheetData>

</xml_diff>